<commit_message>
add output files for 100k variant
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Voltage_3V3_5V/Rev03/100k_pulldown/BOM/BOM_JLC-UZ_D_Voltage_3V3_5V(100k_pulldown_IOs).xlsx
+++ b/Project Outputs for UZ_D_Voltage_3V3_5V/Rev03/100k_pulldown/BOM/BOM_JLC-UZ_D_Voltage_3V3_5V(100k_pulldown_IOs).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ZC\uz_d_voltage_3v3_5v\Project Outputs for UZ_D_Voltage_3V3_5V\Rev03\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\altium\uz_d_voltage_3v3_5v\Project Outputs for UZ_D_Voltage_3V3_5V\Rev03\100k_pulldown\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7960293-B098-42DA-AC0E-BFF2DEC37956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D63C3F-B158-44AC-86DE-CF989D8A4AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2282" yWindow="2282" windowWidth="29086" windowHeight="13640" xr2:uid="{06DCD9D0-4B97-453A-B2BB-0D412038D46E}"/>
+    <workbookView xWindow="-5145" yWindow="-20865" windowWidth="38700" windowHeight="15105" xr2:uid="{669A8D5C-6CD1-4340-B93D-D10A896BF435}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_D_Voltage_3V3_5V(100" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="174">
   <si>
     <t>Quantity</t>
   </si>
@@ -240,7 +240,7 @@
     <t>100k</t>
   </si>
   <si>
-    <t>R6, R7, R42, R73, R74, R85, R86, R87, R88, R89, R90, R91, R92, R93, R94, R95, R96, R97, R98, R99, R100, R101, R102, R103, R104, R105, R106, R107, R108, R109, R110, R111</t>
+    <t>R6, R7</t>
   </si>
   <si>
     <t>UZgen_R_0603_100k</t>
@@ -276,6 +276,9 @@
     <t>UZgen_R_0603_39R</t>
   </si>
   <si>
+    <t>R42, R73, R74, R85, R86, R87, R88, R89, R90, R91, R92, R93, R94, R95, R96, R97, R98, R99, R100, R101, R102, R103, R104, R105, R106, R107, R108, R109, R110, R111</t>
+  </si>
+  <si>
     <t>0R</t>
   </si>
   <si>
@@ -514,6 +517,51 @@
   </si>
   <si>
     <t>IPL1-120-01-XX-D-RA</t>
+  </si>
+  <si>
+    <t>C25804</t>
+  </si>
+  <si>
+    <t>C23162</t>
+  </si>
+  <si>
+    <t>C25803</t>
+  </si>
+  <si>
+    <t>C23154</t>
+  </si>
+  <si>
+    <t>C21189</t>
+  </si>
+  <si>
+    <t>C13167</t>
+  </si>
+  <si>
+    <t>C21190</t>
+  </si>
+  <si>
+    <t>C23025</t>
+  </si>
+  <si>
+    <t>C23182</t>
+  </si>
+  <si>
+    <t>C7423882</t>
+  </si>
+  <si>
+    <t>C7423878</t>
+  </si>
+  <si>
+    <t>C14663</t>
+  </si>
+  <si>
+    <t>C107083</t>
+  </si>
+  <si>
+    <t>C106248</t>
+  </si>
+  <si>
+    <t>C7509499</t>
   </si>
 </sst>
 </file>
@@ -889,23 +937,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1B50E87-CF27-45DE-B40B-B4813A18B938}">
-  <dimension ref="A1:K30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49F85FF4-0F88-4B6B-8F3C-E4C6E6A7A882}">
+  <dimension ref="A1:K31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.375" customWidth="1"/>
-    <col min="2" max="2" width="18.75" customWidth="1"/>
-    <col min="3" max="3" width="17.375" customWidth="1"/>
-    <col min="4" max="4" width="16.25" customWidth="1"/>
-    <col min="5" max="5" width="16.625" customWidth="1"/>
-    <col min="6" max="6" width="16.125" customWidth="1"/>
-    <col min="7" max="7" width="23.875" customWidth="1"/>
-    <col min="8" max="8" width="8.625" customWidth="1"/>
-    <col min="9" max="9" width="9.875" customWidth="1"/>
-    <col min="10" max="11" width="16.25" customWidth="1"/>
+    <col min="1" max="1" width="9.06640625" customWidth="1"/>
+    <col min="2" max="2" width="18.1328125" customWidth="1"/>
+    <col min="3" max="3" width="16.73046875" customWidth="1"/>
+    <col min="4" max="4" width="15.73046875" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="107" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.1328125" customWidth="1"/>
+    <col min="8" max="8" width="7.265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.53125" customWidth="1"/>
+    <col min="10" max="10" width="26.86328125" customWidth="1"/>
+    <col min="11" max="11" width="15.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -940,7 +989,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>12</v>
       </c>
@@ -969,9 +1018,11 @@
       <c r="J2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="1"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K2" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1000,9 +1051,11 @@
       <c r="J3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="1"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K3" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -1031,9 +1084,11 @@
       <c r="J4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="1"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K4" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -1062,7 +1117,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>1</v>
       </c>
@@ -1093,7 +1148,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>3</v>
       </c>
@@ -1126,7 +1181,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -1153,9 +1208,11 @@
       <c r="J8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="K8" s="1"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>2</v>
       </c>
@@ -1186,7 +1243,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>41</v>
       </c>
@@ -1213,9 +1270,11 @@
       <c r="J10" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="K10" s="1"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K10" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>3</v>
       </c>
@@ -1242,11 +1301,13 @@
       <c r="J11" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="K11" s="1"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K11" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>65</v>
@@ -1271,9 +1332,11 @@
       <c r="J12" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K12" s="1"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K12" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>1</v>
       </c>
@@ -1304,7 +1367,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>30</v>
       </c>
@@ -1331,23 +1394,25 @@
       <c r="J14" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="K14" s="1"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K14" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>59</v>
@@ -1358,25 +1423,27 @@
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A16" s="1">
+        <v>2</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="K15" s="1"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <v>1</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>59</v>
@@ -1387,25 +1454,27 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="K16" s="1"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <v>1</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>59</v>
@@ -1416,25 +1485,27 @@
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A18" s="1">
+        <v>1</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="K17" s="1"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>2</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>59</v>
@@ -1445,25 +1516,27 @@
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A19" s="1">
+        <v>2</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="K18" s="1"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>1</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>59</v>
@@ -1474,343 +1547,380 @@
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="K19" s="1"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
         <v>1</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>93</v>
+        <v>60</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K20" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
         <v>1</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="K21" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
         <v>1</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="K22" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="K22" s="2" t="s">
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A23" s="1">
+        <v>1</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>112</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <v>9</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="K23" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="K23" s="2" t="s">
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A24" s="1">
+        <v>9</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>119</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>1</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K24" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="K24" s="2" t="s">
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A25" s="1">
+        <v>1</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>125</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>4</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="K25" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="K25" s="2" t="s">
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A26" s="1">
+        <v>4</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>132</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>1</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>137</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="K26" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A27" s="1">
         <v>1</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E27" s="1"/>
+        <v>129</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="F27" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="K27" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="K27" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A28" s="1">
         <v>1</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>146</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="E28" s="1"/>
       <c r="F28" s="2" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K28" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="K28" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A29" s="1">
         <v>1</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="E29" s="1"/>
+        <v>129</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>147</v>
+      </c>
       <c r="F29" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="K29" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="K29" s="1"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A30" s="1">
         <v>1</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
       <c r="J30" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="K30" s="1"/>
+        <v>150</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A31" s="1">
+        <v>1</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E31" s="1"/>
+      <c r="F31" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>169</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="128" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>